<commit_message>
Remove real catalog and shipment ids from the open-source defaults.
Empty the three mapping files, use the desensitized customs workbook, and replace the sample SKUs and the deshu example shipment id.

Co-authored-by: huangyuehui1998-dev <huangyuehui1998-dev@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend/templates/customs/报关资料模板.xlsx
+++ b/backend/templates/customs/报关资料模板.xlsx
@@ -859,11 +859,7 @@
           <t>境内发货人</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>91420113MACWNNKU99</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>出境关别</t>
@@ -879,9 +875,7 @@
           <t>出口日期</t>
         </is>
       </c>
-      <c r="H3" s="7" t="n">
-        <v>46198</v>
-      </c>
+      <c r="H3" s="7" t="n"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>申报日期</t>
@@ -911,7 +905,7 @@
     <row r="4" ht="17.1" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
@@ -982,7 +976,7 @@
       </c>
       <c r="V5" s="8" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="W5" s="8" t="inlineStr"/>
@@ -1024,11 +1018,7 @@
           <t>生产销售单位</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>91420113MACWNNKU99</t>
-        </is>
-      </c>
+      <c r="C7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>监管方式</t>
@@ -1077,7 +1067,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -1164,7 +1154,7 @@
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1289,13 +1279,9 @@
           <t>纸箱</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
-        <v>115</v>
-      </c>
+      <c r="E12" s="18" t="n"/>
       <c r="F12" s="18" t="inlineStr"/>
-      <c r="G12" s="18" t="n">
-        <v>661.4</v>
-      </c>
+      <c r="G12" s="18" t="n"/>
       <c r="I12" s="18" t="inlineStr">
         <is>
           <t>C&amp;F</t>
@@ -1334,7 +1320,7 @@
       </c>
       <c r="W13" s="6" t="inlineStr">
         <is>
-          <t>非互认国家（地区）AEO企业等其他情形，编码免于填报。对于AEO互认国家（地区）企业的，编码填报AEO编码，填报样式按照海关总署发布的相关公告要求填报（如新加坡AEO企业填报样式为：SG123456789012，韩国AEO企业填报样式为KR1234567，具体见相关公告要求）。</t>
+          <t>非互认国家（地区）AEO企业等其他情形，编码免于填报。对于AEO互认国家（地区）企业的，编码填报AEO编码，填报样式按照海关总署发布的相关公告要求填报（如新加坡AEO企业填报样式为：DEMO-ORDER，韩国AEO企业填报样式为DEMO-ORDER，具体见相关公告要求）。</t>
         </is>
       </c>
       <c r="X13" s="6" t="inlineStr"/>
@@ -1392,7 +1378,7 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>订单编号：JUS7HB115。仓库编码：VGT2，SCK4，IND9，PSP3，AVP1。FBA编码：FBA19GVFX5SC，FBA19GVDVGS5，FBA19GVFCZ70，FBA19GVD3PNH，FBA19GVF02NV。</t>
+          <t>订单编号：DEMO-ORDER。仓库编码：DEMO，DEMO，DEMO，DEMO，DEMO。FBA编码：FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO。</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
@@ -1531,31 +1517,21 @@
       <c r="AB19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="23" customHeight="1">
-      <c r="A20" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="26" t="n">
-        <v>6307909000</v>
-      </c>
+      <c r="A20" s="27" t="n"/>
+      <c r="B20" s="26" t="n"/>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="G20" s="26" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="n"/>
       <c r="H20" s="26" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="I20" s="10" t="n">
-        <v>35.51</v>
-      </c>
-      <c r="J20" s="10" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="10" t="n"/>
       <c r="K20" s="27" t="inlineStr">
         <is>
           <t>中国</t>
@@ -1571,7 +1547,7 @@
       <c r="O20" s="27" t="inlineStr"/>
       <c r="P20" s="27" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>示例城市</t>
         </is>
       </c>
       <c r="Q20" s="27" t="inlineStr"/>
@@ -1758,14 +1734,10 @@
           <t>总计</t>
         </is>
       </c>
-      <c r="G27" s="26" t="n">
-        <v>460</v>
-      </c>
+      <c r="G27" s="26" t="n"/>
       <c r="H27" s="26" t="inlineStr"/>
       <c r="I27" s="26" t="inlineStr"/>
-      <c r="J27" s="18" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="J27" s="18" t="n"/>
       <c r="K27" s="26" t="inlineStr"/>
       <c r="T27" s="26" t="inlineStr"/>
       <c r="U27" s="26" t="inlineStr"/>
@@ -1858,8 +1830,8 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="P19:R19"/>
     <mergeCell ref="L9:N9"/>
+    <mergeCell ref="L18:S18"/>
     <mergeCell ref="H3:J3"/>
-    <mergeCell ref="L18:S18"/>
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="A1:S1"/>
@@ -2697,21 +2669,17 @@
       </c>
     </row>
     <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="32" t="n">
-        <v>1</v>
-      </c>
+      <c r="A10" s="32" t="n"/>
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="C10" s="32" t="n">
-        <v>6307909000</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="n"/>
       <c r="D10" s="32" t="inlineStr"/>
       <c r="E10" s="32" t="inlineStr">
         <is>
-          <t>JoyBlooms</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="F10" s="32" t="inlineStr">
@@ -2731,49 +2699,25 @@
       </c>
       <c r="I10" s="32" t="inlineStr">
         <is>
-          <t>1|2|宠物用|品牌：JoyBlooms牌|型号：无型号</t>
+          <t>1|2|宠物用|品牌：DEMO牌|型号：无型号</t>
         </is>
       </c>
     </row>
     <row r="11" ht="27" customHeight="1">
-      <c r="A11" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A11" s="32" t="n"/>
+      <c r="B11" s="32" t="n"/>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="32" t="n"/>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="32" t="n"/>
+      <c r="H11" s="32" t="n"/>
+      <c r="I11" s="32" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A12" s="32" t="n"/>
+      <c r="B12" s="32" t="n"/>
+      <c r="C12" s="32" t="n"/>
       <c r="D12" s="32" t="inlineStr"/>
       <c r="E12" s="32" t="inlineStr"/>
       <c r="F12" s="32" t="inlineStr"/>
@@ -2782,15 +2726,9 @@
       <c r="I12" s="32" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A13" s="32" t="n"/>
+      <c r="B13" s="32" t="n"/>
+      <c r="C13" s="32" t="n"/>
       <c r="D13" s="32" t="inlineStr"/>
       <c r="E13" s="32" t="inlineStr"/>
       <c r="F13" s="32" t="inlineStr"/>
@@ -2799,15 +2737,9 @@
       <c r="I13" s="32" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A14" s="32" t="n"/>
+      <c r="B14" s="32" t="n"/>
+      <c r="C14" s="32" t="n"/>
       <c r="D14" s="32" t="inlineStr"/>
       <c r="E14" s="32" t="inlineStr"/>
       <c r="F14" s="32" t="inlineStr"/>
@@ -2816,15 +2748,9 @@
       <c r="I14" s="32" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="32" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A15" s="32" t="n"/>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="32" t="n"/>
       <c r="D15" s="32" t="inlineStr"/>
       <c r="E15" s="32" t="inlineStr"/>
       <c r="F15" s="32" t="inlineStr"/>
@@ -2913,7 +2839,7 @@
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
     </row>
@@ -2935,9 +2861,7 @@
 DATE:</t>
         </is>
       </c>
-      <c r="G3" s="37" t="n">
-        <v>46198</v>
-      </c>
+      <c r="G3" s="37" t="n"/>
     </row>
     <row r="4" ht="27.95" customHeight="1">
       <c r="A4" s="22" t="inlineStr"/>
@@ -3012,23 +2936,17 @@
       </c>
       <c r="C8" s="38" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n"/>
       <c r="E8" s="17" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="F8" s="17" t="n">
-        <v>35.51</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="32" t="inlineStr">
@@ -3036,19 +2954,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C9" s="38" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
       <c r="F9" s="17" t="inlineStr"/>
-      <c r="G9" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="32" t="inlineStr">
@@ -3056,19 +2966,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C10" s="38" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
       <c r="F10" s="17" t="inlineStr"/>
-      <c r="G10" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="32" t="inlineStr">
@@ -3076,19 +2978,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C11" s="38" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
       <c r="F11" s="17" t="inlineStr"/>
-      <c r="G11" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="32" t="inlineStr">
@@ -3096,19 +2990,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C12" s="38" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
       <c r="F12" s="17" t="inlineStr"/>
-      <c r="G12" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="32" t="inlineStr">
@@ -3116,19 +3002,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C13" s="38" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
       <c r="F13" s="17" t="inlineStr"/>
-      <c r="G13" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="32" t="inlineStr"/>
@@ -3144,17 +3022,13 @@
           <t>  </t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C15" s="17" t="n"/>
       <c r="F15" s="17" t="inlineStr">
         <is>
           <t>总计TOTAL:</t>
         </is>
       </c>
-      <c r="G15" s="17" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="G15" s="17" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="32" t="inlineStr">
@@ -3325,9 +3199,7 @@
 Date：</t>
         </is>
       </c>
-      <c r="G2" s="41" t="n">
-        <v>46198</v>
-      </c>
+      <c r="G2" s="41" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="42" t="inlineStr"/>
@@ -3343,7 +3215,7 @@
       </c>
       <c r="G3" s="46" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3239,7 @@
       </c>
       <c r="G4" s="46" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
     </row>
@@ -3464,97 +3336,61 @@
       <c r="A9" s="30" t="inlineStr"/>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="C9" s="52" t="n">
-        <v>115</v>
-      </c>
-      <c r="D9" s="52" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="C9" s="52" t="n"/>
+      <c r="D9" s="52" t="n"/>
       <c r="E9" s="52" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
       <c r="F9" s="25" t="inlineStr"/>
-      <c r="G9" s="25" t="n">
-        <v>661.4</v>
-      </c>
+      <c r="G9" s="25" t="n"/>
       <c r="H9" s="53" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B10" s="52" t="n"/>
       <c r="C10" s="54" t="inlineStr"/>
-      <c r="D10" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D10" s="52" t="n"/>
+      <c r="E10" s="52" t="n"/>
       <c r="F10" s="25" t="inlineStr"/>
       <c r="G10" s="25" t="inlineStr"/>
       <c r="H10" s="53" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B11" s="52" t="n"/>
       <c r="C11" s="52" t="inlineStr"/>
-      <c r="D11" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D11" s="52" t="n"/>
+      <c r="E11" s="52" t="n"/>
       <c r="F11" s="18" t="inlineStr"/>
       <c r="G11" s="18" t="inlineStr"/>
       <c r="H11" s="53" t="inlineStr"/>
     </row>
     <row r="12" ht="66" customHeight="1">
-      <c r="B12" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B12" s="52" t="n"/>
       <c r="C12" s="52" t="inlineStr"/>
-      <c r="D12" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D12" s="52" t="n"/>
+      <c r="E12" s="52" t="n"/>
       <c r="F12" s="18" t="inlineStr"/>
       <c r="G12" s="18" t="inlineStr"/>
       <c r="H12" s="53" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B13" s="52" t="n"/>
       <c r="C13" s="52" t="inlineStr"/>
-      <c r="D13" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D13" s="52" t="n"/>
+      <c r="E13" s="52" t="n"/>
       <c r="F13" s="18" t="inlineStr"/>
       <c r="G13" s="18" t="inlineStr"/>
       <c r="H13" s="53" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B14" s="52" t="n"/>
       <c r="C14" s="52" t="inlineStr"/>
-      <c r="D14" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D14" s="52" t="n"/>
+      <c r="E14" s="52" t="n"/>
       <c r="F14" s="18" t="inlineStr"/>
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="53" t="inlineStr"/>
@@ -3567,17 +3403,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr"/>
-      <c r="C15" s="42" t="n">
-        <v>115</v>
-      </c>
-      <c r="D15" s="52" t="n">
-        <v>460</v>
-      </c>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="52" t="n"/>
       <c r="E15" s="52" t="inlineStr"/>
       <c r="F15" s="42" t="inlineStr"/>
-      <c r="G15" s="42" t="n">
-        <v>661.4</v>
-      </c>
+      <c r="G15" s="42" t="n"/>
     </row>
     <row r="16" ht="18.95" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
@@ -3744,7 +3574,7 @@
       </c>
       <c r="B2" s="57" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="E2" s="58" t="inlineStr"/>
@@ -3797,9 +3627,7 @@
           <t>传  真</t>
         </is>
       </c>
-      <c r="D6" s="65" t="n">
-        <v>0</v>
-      </c>
+      <c r="D6" s="65" t="n"/>
       <c r="E6" s="60" t="inlineStr">
         <is>
           <t>Contract No:</t>
@@ -3807,7 +3635,7 @@
       </c>
       <c r="F6" s="66" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
       <c r="I6" s="42" t="inlineStr"/>
@@ -3847,9 +3675,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="F8" s="69" t="n">
-        <v>46198</v>
-      </c>
+      <c r="F8" s="69" t="n"/>
     </row>
     <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="56" t="inlineStr">
@@ -3873,7 +3699,7 @@
       </c>
       <c r="B10" s="71" t="inlineStr">
         <is>
-          <t>订单编号：JUS7HB115。仓库编码：VGT2，SCK4，IND9，PSP3，AVP1。FBA编码：FBA19GVFX5SC，FBA19GVDVGS5，FBA19GVFCZ70，FBA19GVD3PNH，FBA19GVF02NV。</t>
+          <t>订单编号：DEMO-ORDER。仓库编码：DEMO，DEMO，DEMO，DEMO，DEMO。FBA编码：FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO。</t>
         </is>
       </c>
       <c r="E10" s="60" t="inlineStr">
@@ -3883,7 +3709,7 @@
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>示例城市</t>
         </is>
       </c>
     </row>
@@ -3911,17 +3737,13 @@
           <t>电   话</t>
         </is>
       </c>
-      <c r="B12" s="56" t="n">
-        <v>0</v>
-      </c>
+      <c r="B12" s="56" t="n"/>
       <c r="C12" s="63" t="inlineStr">
         <is>
           <t>传  真</t>
         </is>
       </c>
-      <c r="D12" s="59" t="n">
-        <v>0</v>
-      </c>
+      <c r="D12" s="59" t="n"/>
     </row>
     <row r="13" ht="14.1" customHeight="1">
       <c r="A13" s="67" t="inlineStr">
@@ -4015,23 +3837,17 @@
     <row r="18" ht="29" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="n"/>
       <c r="D18" s="26" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="E18" s="26" t="n">
-        <v>35.51</v>
-      </c>
-      <c r="F18" s="26" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="26" t="n"/>
       <c r="G18" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4039,21 +3855,11 @@
       </c>
     </row>
     <row r="19" ht="29" customHeight="1">
-      <c r="A19" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A19" s="28" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="26" t="n"/>
       <c r="G19" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4061,21 +3867,11 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A20" s="28" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="26" t="n"/>
+      <c r="F20" s="26" t="n"/>
       <c r="G20" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4083,21 +3879,11 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A21" s="28" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="26" t="n"/>
+      <c r="F21" s="26" t="n"/>
       <c r="G21" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4105,21 +3891,11 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A22" s="28" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
       <c r="G22" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4127,21 +3903,11 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A23" s="28" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="26" t="n"/>
+      <c r="E23" s="26" t="n"/>
+      <c r="F23" s="26" t="n"/>
       <c r="G23" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4154,18 +3920,14 @@
           <t>合计：</t>
         </is>
       </c>
-      <c r="C24" s="26" t="n">
-        <v>460</v>
-      </c>
+      <c r="C24" s="26" t="n"/>
       <c r="D24" s="26" t="inlineStr"/>
       <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Total Amount:</t>
         </is>
       </c>
-      <c r="F24" s="26" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="F24" s="26" t="n"/>
       <c r="G24" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4204,9 +3966,7 @@
           <t>  </t>
         </is>
       </c>
-      <c r="D27" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="D27" s="21" t="n"/>
       <c r="H27" s="21" t="inlineStr"/>
     </row>
     <row r="28" ht="13.5" customHeight="1">
@@ -4271,9 +4031,7 @@
           <t>Time of Shipment:</t>
         </is>
       </c>
-      <c r="B32" s="77" t="n">
-        <v>46213</v>
-      </c>
+      <c r="B32" s="77" t="n"/>
       <c r="D32" s="21" t="inlineStr">
         <is>
           <t>之前</t>
@@ -4457,7 +4215,7 @@
       </c>
       <c r="E43" s="51" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="G43" s="51" t="inlineStr"/>
@@ -4484,9 +4242,9 @@
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="B4:D5"/>
     <mergeCell ref="F17:H17"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="F3:H3"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G23:H23"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G19:H19"/>
@@ -4561,14 +4319,10 @@
           <t>编号：</t>
         </is>
       </c>
-      <c r="H5" s="21" t="n">
-        <v>4403180086</v>
-      </c>
+      <c r="H5" s="21" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="C6" s="29" t="n">
-        <v>0</v>
-      </c>
+      <c r="C6" s="29" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
@@ -4613,7 +4367,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>2022 年 12 月 31日止。</t>
+          <t xml:space="preserve">    年  月  日止。</t>
         </is>
       </c>
     </row>
@@ -4633,9 +4387,7 @@
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="H16" s="81" t="n">
-        <v>46197</v>
-      </c>
+      <c r="H16" s="81" t="n"/>
     </row>
     <row r="17"/>
     <row r="18" ht="18.75" customHeight="1">
@@ -4661,7 +4413,7 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -4670,9 +4422,7 @@
           <t>被委托方</t>
         </is>
       </c>
-      <c r="H21" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="H21" s="5" t="n"/>
     </row>
     <row r="22" ht="27" customHeight="1">
       <c r="B22" s="5" t="inlineStr">
@@ -4682,7 +4432,7 @@
       </c>
       <c r="C22" s="38" t="inlineStr">
         <is>
-          <t>宠物垫</t>
+          <t>示例商品</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr"/>
@@ -4699,18 +4449,14 @@
           <t>HS编码</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
-        <v>6307909000</v>
-      </c>
+      <c r="C23" s="17" t="n"/>
       <c r="F23" s="6" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
           <t>收到单证日期</t>
         </is>
       </c>
-      <c r="H23" s="82" t="n">
-        <v>46198</v>
-      </c>
+      <c r="H23" s="82" t="n"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="B24" s="5" t="inlineStr">
@@ -4718,9 +4464,7 @@
           <t>货物总价</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="C24" s="17" t="n"/>
       <c r="F24" s="6" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
@@ -4744,9 +4488,7 @@
           <t>进出口日期</t>
         </is>
       </c>
-      <c r="C25" s="83" t="n">
-        <v>46199</v>
-      </c>
+      <c r="C25" s="83" t="n"/>
       <c r="F25" s="6" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
@@ -4804,7 +4546,7 @@
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>示例城市</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr"/>
@@ -4995,18 +4737,14 @@
       </c>
       <c r="C45" s="22" t="inlineStr"/>
       <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="86" t="n">
-        <v>46197</v>
-      </c>
+      <c r="E45" s="86" t="n"/>
       <c r="G45" s="6" t="inlineStr">
         <is>
           <t>联系电话：</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr"/>
-      <c r="I45" s="82" t="n">
-        <v>46198</v>
-      </c>
+      <c r="I45" s="82" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="B46" s="22" t="inlineStr"/>

</xml_diff>

<commit_message>
V4 phase A/B + OSS docs/desensitization (#14)
Offline Univer preview, carton return, Lingxing import; open-source docs; strip secrets and real listing defaults from current tree.
</commit_message>
<xml_diff>
--- a/backend/templates/customs/报关资料模板.xlsx
+++ b/backend/templates/customs/报关资料模板.xlsx
@@ -859,11 +859,7 @@
           <t>境内发货人</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>91420113MACWNNKU99</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>出境关别</t>
@@ -879,9 +875,7 @@
           <t>出口日期</t>
         </is>
       </c>
-      <c r="H3" s="7" t="n">
-        <v>46198</v>
-      </c>
+      <c r="H3" s="7" t="n"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>申报日期</t>
@@ -911,7 +905,7 @@
     <row r="4" ht="17.1" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
@@ -982,7 +976,7 @@
       </c>
       <c r="V5" s="8" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="W5" s="8" t="inlineStr"/>
@@ -1024,11 +1018,7 @@
           <t>生产销售单位</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>91420113MACWNNKU99</t>
-        </is>
-      </c>
+      <c r="C7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>监管方式</t>
@@ -1077,7 +1067,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -1164,7 +1154,7 @@
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1289,13 +1279,9 @@
           <t>纸箱</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
-        <v>115</v>
-      </c>
+      <c r="E12" s="18" t="n"/>
       <c r="F12" s="18" t="inlineStr"/>
-      <c r="G12" s="18" t="n">
-        <v>661.4</v>
-      </c>
+      <c r="G12" s="18" t="n"/>
       <c r="I12" s="18" t="inlineStr">
         <is>
           <t>C&amp;F</t>
@@ -1334,7 +1320,7 @@
       </c>
       <c r="W13" s="6" t="inlineStr">
         <is>
-          <t>非互认国家（地区）AEO企业等其他情形，编码免于填报。对于AEO互认国家（地区）企业的，编码填报AEO编码，填报样式按照海关总署发布的相关公告要求填报（如新加坡AEO企业填报样式为：SG123456789012，韩国AEO企业填报样式为KR1234567，具体见相关公告要求）。</t>
+          <t>非互认国家（地区）AEO企业等其他情形，编码免于填报。对于AEO互认国家（地区）企业的，编码填报AEO编码，填报样式按照海关总署发布的相关公告要求填报（如新加坡AEO企业填报样式为：DEMO-ORDER，韩国AEO企业填报样式为DEMO-ORDER，具体见相关公告要求）。</t>
         </is>
       </c>
       <c r="X13" s="6" t="inlineStr"/>
@@ -1392,7 +1378,7 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>订单编号：JUS7HB115。仓库编码：VGT2，SCK4，IND9，PSP3，AVP1。FBA编码：FBA19GVFX5SC，FBA19GVDVGS5，FBA19GVFCZ70，FBA19GVD3PNH，FBA19GVF02NV。</t>
+          <t>订单编号：DEMO-ORDER。仓库编码：DEMO，DEMO，DEMO，DEMO，DEMO。FBA编码：FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO。</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
@@ -1531,31 +1517,21 @@
       <c r="AB19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="23" customHeight="1">
-      <c r="A20" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="26" t="n">
-        <v>6307909000</v>
-      </c>
+      <c r="A20" s="27" t="n"/>
+      <c r="B20" s="26" t="n"/>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="G20" s="26" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="n"/>
       <c r="H20" s="26" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="I20" s="10" t="n">
-        <v>35.51</v>
-      </c>
-      <c r="J20" s="10" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="10" t="n"/>
       <c r="K20" s="27" t="inlineStr">
         <is>
           <t>中国</t>
@@ -1571,7 +1547,7 @@
       <c r="O20" s="27" t="inlineStr"/>
       <c r="P20" s="27" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>示例城市</t>
         </is>
       </c>
       <c r="Q20" s="27" t="inlineStr"/>
@@ -1758,14 +1734,10 @@
           <t>总计</t>
         </is>
       </c>
-      <c r="G27" s="26" t="n">
-        <v>460</v>
-      </c>
+      <c r="G27" s="26" t="n"/>
       <c r="H27" s="26" t="inlineStr"/>
       <c r="I27" s="26" t="inlineStr"/>
-      <c r="J27" s="18" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="J27" s="18" t="n"/>
       <c r="K27" s="26" t="inlineStr"/>
       <c r="T27" s="26" t="inlineStr"/>
       <c r="U27" s="26" t="inlineStr"/>
@@ -1858,8 +1830,8 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="P19:R19"/>
     <mergeCell ref="L9:N9"/>
+    <mergeCell ref="L18:S18"/>
     <mergeCell ref="H3:J3"/>
-    <mergeCell ref="L18:S18"/>
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="A1:S1"/>
@@ -2697,21 +2669,17 @@
       </c>
     </row>
     <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="32" t="n">
-        <v>1</v>
-      </c>
+      <c r="A10" s="32" t="n"/>
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="C10" s="32" t="n">
-        <v>6307909000</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="n"/>
       <c r="D10" s="32" t="inlineStr"/>
       <c r="E10" s="32" t="inlineStr">
         <is>
-          <t>JoyBlooms</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="F10" s="32" t="inlineStr">
@@ -2731,49 +2699,25 @@
       </c>
       <c r="I10" s="32" t="inlineStr">
         <is>
-          <t>1|2|宠物用|品牌：JoyBlooms牌|型号：无型号</t>
+          <t>1|2|宠物用|品牌：DEMO牌|型号：无型号</t>
         </is>
       </c>
     </row>
     <row r="11" ht="27" customHeight="1">
-      <c r="A11" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A11" s="32" t="n"/>
+      <c r="B11" s="32" t="n"/>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="32" t="n"/>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="32" t="n"/>
+      <c r="H11" s="32" t="n"/>
+      <c r="I11" s="32" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A12" s="32" t="n"/>
+      <c r="B12" s="32" t="n"/>
+      <c r="C12" s="32" t="n"/>
       <c r="D12" s="32" t="inlineStr"/>
       <c r="E12" s="32" t="inlineStr"/>
       <c r="F12" s="32" t="inlineStr"/>
@@ -2782,15 +2726,9 @@
       <c r="I12" s="32" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A13" s="32" t="n"/>
+      <c r="B13" s="32" t="n"/>
+      <c r="C13" s="32" t="n"/>
       <c r="D13" s="32" t="inlineStr"/>
       <c r="E13" s="32" t="inlineStr"/>
       <c r="F13" s="32" t="inlineStr"/>
@@ -2799,15 +2737,9 @@
       <c r="I13" s="32" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A14" s="32" t="n"/>
+      <c r="B14" s="32" t="n"/>
+      <c r="C14" s="32" t="n"/>
       <c r="D14" s="32" t="inlineStr"/>
       <c r="E14" s="32" t="inlineStr"/>
       <c r="F14" s="32" t="inlineStr"/>
@@ -2816,15 +2748,9 @@
       <c r="I14" s="32" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="32" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="32" t="n">
-        <v>0</v>
-      </c>
+      <c r="A15" s="32" t="n"/>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="32" t="n"/>
       <c r="D15" s="32" t="inlineStr"/>
       <c r="E15" s="32" t="inlineStr"/>
       <c r="F15" s="32" t="inlineStr"/>
@@ -2913,7 +2839,7 @@
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
     </row>
@@ -2935,9 +2861,7 @@
 DATE:</t>
         </is>
       </c>
-      <c r="G3" s="37" t="n">
-        <v>46198</v>
-      </c>
+      <c r="G3" s="37" t="n"/>
     </row>
     <row r="4" ht="27.95" customHeight="1">
       <c r="A4" s="22" t="inlineStr"/>
@@ -3012,23 +2936,17 @@
       </c>
       <c r="C8" s="38" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n"/>
       <c r="E8" s="17" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="F8" s="17" t="n">
-        <v>35.51</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="32" t="inlineStr">
@@ -3036,19 +2954,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C9" s="38" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
       <c r="F9" s="17" t="inlineStr"/>
-      <c r="G9" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="32" t="inlineStr">
@@ -3056,19 +2966,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C10" s="38" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
       <c r="F10" s="17" t="inlineStr"/>
-      <c r="G10" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="32" t="inlineStr">
@@ -3076,19 +2978,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C11" s="38" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
       <c r="F11" s="17" t="inlineStr"/>
-      <c r="G11" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="32" t="inlineStr">
@@ -3096,19 +2990,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C12" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C12" s="38" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
       <c r="F12" s="17" t="inlineStr"/>
-      <c r="G12" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="32" t="inlineStr">
@@ -3116,19 +3002,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C13" s="38" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
       <c r="F13" s="17" t="inlineStr"/>
-      <c r="G13" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="32" t="inlineStr"/>
@@ -3144,17 +3022,13 @@
           <t>  </t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
-        <v>0</v>
-      </c>
+      <c r="C15" s="17" t="n"/>
       <c r="F15" s="17" t="inlineStr">
         <is>
           <t>总计TOTAL:</t>
         </is>
       </c>
-      <c r="G15" s="17" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="G15" s="17" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="32" t="inlineStr">
@@ -3325,9 +3199,7 @@
 Date：</t>
         </is>
       </c>
-      <c r="G2" s="41" t="n">
-        <v>46198</v>
-      </c>
+      <c r="G2" s="41" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="42" t="inlineStr"/>
@@ -3343,7 +3215,7 @@
       </c>
       <c r="G3" s="46" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3239,7 @@
       </c>
       <c r="G4" s="46" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
     </row>
@@ -3464,97 +3336,61 @@
       <c r="A9" s="30" t="inlineStr"/>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="C9" s="52" t="n">
-        <v>115</v>
-      </c>
-      <c r="D9" s="52" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="C9" s="52" t="n"/>
+      <c r="D9" s="52" t="n"/>
       <c r="E9" s="52" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
       <c r="F9" s="25" t="inlineStr"/>
-      <c r="G9" s="25" t="n">
-        <v>661.4</v>
-      </c>
+      <c r="G9" s="25" t="n"/>
       <c r="H9" s="53" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B10" s="52" t="n"/>
       <c r="C10" s="54" t="inlineStr"/>
-      <c r="D10" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D10" s="52" t="n"/>
+      <c r="E10" s="52" t="n"/>
       <c r="F10" s="25" t="inlineStr"/>
       <c r="G10" s="25" t="inlineStr"/>
       <c r="H10" s="53" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B11" s="52" t="n"/>
       <c r="C11" s="52" t="inlineStr"/>
-      <c r="D11" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D11" s="52" t="n"/>
+      <c r="E11" s="52" t="n"/>
       <c r="F11" s="18" t="inlineStr"/>
       <c r="G11" s="18" t="inlineStr"/>
       <c r="H11" s="53" t="inlineStr"/>
     </row>
     <row r="12" ht="66" customHeight="1">
-      <c r="B12" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B12" s="52" t="n"/>
       <c r="C12" s="52" t="inlineStr"/>
-      <c r="D12" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D12" s="52" t="n"/>
+      <c r="E12" s="52" t="n"/>
       <c r="F12" s="18" t="inlineStr"/>
       <c r="G12" s="18" t="inlineStr"/>
       <c r="H12" s="53" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B13" s="52" t="n"/>
       <c r="C13" s="52" t="inlineStr"/>
-      <c r="D13" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D13" s="52" t="n"/>
+      <c r="E13" s="52" t="n"/>
       <c r="F13" s="18" t="inlineStr"/>
       <c r="G13" s="18" t="inlineStr"/>
       <c r="H13" s="53" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B14" s="52" t="n"/>
       <c r="C14" s="52" t="inlineStr"/>
-      <c r="D14" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D14" s="52" t="n"/>
+      <c r="E14" s="52" t="n"/>
       <c r="F14" s="18" t="inlineStr"/>
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="53" t="inlineStr"/>
@@ -3567,17 +3403,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr"/>
-      <c r="C15" s="42" t="n">
-        <v>115</v>
-      </c>
-      <c r="D15" s="52" t="n">
-        <v>460</v>
-      </c>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="52" t="n"/>
       <c r="E15" s="52" t="inlineStr"/>
       <c r="F15" s="42" t="inlineStr"/>
-      <c r="G15" s="42" t="n">
-        <v>661.4</v>
-      </c>
+      <c r="G15" s="42" t="n"/>
     </row>
     <row r="16" ht="18.95" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
@@ -3744,7 +3574,7 @@
       </c>
       <c r="B2" s="57" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="E2" s="58" t="inlineStr"/>
@@ -3797,9 +3627,7 @@
           <t>传  真</t>
         </is>
       </c>
-      <c r="D6" s="65" t="n">
-        <v>0</v>
-      </c>
+      <c r="D6" s="65" t="n"/>
       <c r="E6" s="60" t="inlineStr">
         <is>
           <t>Contract No:</t>
@@ -3807,7 +3635,7 @@
       </c>
       <c r="F6" s="66" t="inlineStr">
         <is>
-          <t>JUS7HB115</t>
+          <t>DEMO-ORDER</t>
         </is>
       </c>
       <c r="I6" s="42" t="inlineStr"/>
@@ -3847,9 +3675,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="F8" s="69" t="n">
-        <v>46198</v>
-      </c>
+      <c r="F8" s="69" t="n"/>
     </row>
     <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="56" t="inlineStr">
@@ -3873,7 +3699,7 @@
       </c>
       <c r="B10" s="71" t="inlineStr">
         <is>
-          <t>订单编号：JUS7HB115。仓库编码：VGT2，SCK4，IND9，PSP3，AVP1。FBA编码：FBA19GVFX5SC，FBA19GVDVGS5，FBA19GVFCZ70，FBA19GVD3PNH，FBA19GVF02NV。</t>
+          <t>订单编号：DEMO-ORDER。仓库编码：DEMO，DEMO，DEMO，DEMO，DEMO。FBA编码：FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO，FBA-DEMO。</t>
         </is>
       </c>
       <c r="E10" s="60" t="inlineStr">
@@ -3883,7 +3709,7 @@
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>示例城市</t>
         </is>
       </c>
     </row>
@@ -3911,17 +3737,13 @@
           <t>电   话</t>
         </is>
       </c>
-      <c r="B12" s="56" t="n">
-        <v>0</v>
-      </c>
+      <c r="B12" s="56" t="n"/>
       <c r="C12" s="63" t="inlineStr">
         <is>
           <t>传  真</t>
         </is>
       </c>
-      <c r="D12" s="59" t="n">
-        <v>0</v>
-      </c>
+      <c r="D12" s="59" t="n"/>
     </row>
     <row r="13" ht="14.1" customHeight="1">
       <c r="A13" s="67" t="inlineStr">
@@ -4015,23 +3837,17 @@
     <row r="18" ht="29" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>宠物垫</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="n">
-        <v>460</v>
-      </c>
+          <t>示例商品</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="n"/>
       <c r="D18" s="26" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="E18" s="26" t="n">
-        <v>35.51</v>
-      </c>
-      <c r="F18" s="26" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="26" t="n"/>
       <c r="G18" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4039,21 +3855,11 @@
       </c>
     </row>
     <row r="19" ht="29" customHeight="1">
-      <c r="A19" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A19" s="28" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="26" t="n"/>
       <c r="G19" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4061,21 +3867,11 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A20" s="28" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="26" t="n"/>
+      <c r="F20" s="26" t="n"/>
       <c r="G20" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4083,21 +3879,11 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A21" s="28" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="26" t="n"/>
+      <c r="F21" s="26" t="n"/>
       <c r="G21" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4105,21 +3891,11 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A22" s="28" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
       <c r="G22" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4127,21 +3903,11 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="A23" s="28" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="26" t="n"/>
+      <c r="E23" s="26" t="n"/>
+      <c r="F23" s="26" t="n"/>
       <c r="G23" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4154,18 +3920,14 @@
           <t>合计：</t>
         </is>
       </c>
-      <c r="C24" s="26" t="n">
-        <v>460</v>
-      </c>
+      <c r="C24" s="26" t="n"/>
       <c r="D24" s="26" t="inlineStr"/>
       <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Total Amount:</t>
         </is>
       </c>
-      <c r="F24" s="26" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="F24" s="26" t="n"/>
       <c r="G24" s="26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4204,9 +3966,7 @@
           <t>  </t>
         </is>
       </c>
-      <c r="D27" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="D27" s="21" t="n"/>
       <c r="H27" s="21" t="inlineStr"/>
     </row>
     <row r="28" ht="13.5" customHeight="1">
@@ -4271,9 +4031,7 @@
           <t>Time of Shipment:</t>
         </is>
       </c>
-      <c r="B32" s="77" t="n">
-        <v>46213</v>
-      </c>
+      <c r="B32" s="77" t="n"/>
       <c r="D32" s="21" t="inlineStr">
         <is>
           <t>之前</t>
@@ -4457,7 +4215,7 @@
       </c>
       <c r="E43" s="51" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="G43" s="51" t="inlineStr"/>
@@ -4484,9 +4242,9 @@
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="B4:D5"/>
     <mergeCell ref="F17:H17"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="F3:H3"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G23:H23"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G19:H19"/>
@@ -4561,14 +4319,10 @@
           <t>编号：</t>
         </is>
       </c>
-      <c r="H5" s="21" t="n">
-        <v>4403180086</v>
-      </c>
+      <c r="H5" s="21" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="C6" s="29" t="n">
-        <v>0</v>
-      </c>
+      <c r="C6" s="29" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
@@ -4613,7 +4367,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>2022 年 12 月 31日止。</t>
+          <t xml:space="preserve">    年  月  日止。</t>
         </is>
       </c>
     </row>
@@ -4633,9 +4387,7 @@
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="H16" s="81" t="n">
-        <v>46197</v>
-      </c>
+      <c r="H16" s="81" t="n"/>
     </row>
     <row r="17"/>
     <row r="18" ht="18.75" customHeight="1">
@@ -4661,7 +4413,7 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>武汉花屿森电子商务有限公司</t>
+          <t>示例公司（请在出口商档案里填写）</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -4670,9 +4422,7 @@
           <t>被委托方</t>
         </is>
       </c>
-      <c r="H21" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="H21" s="5" t="n"/>
     </row>
     <row r="22" ht="27" customHeight="1">
       <c r="B22" s="5" t="inlineStr">
@@ -4682,7 +4432,7 @@
       </c>
       <c r="C22" s="38" t="inlineStr">
         <is>
-          <t>宠物垫</t>
+          <t>示例商品</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr"/>
@@ -4699,18 +4449,14 @@
           <t>HS编码</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
-        <v>6307909000</v>
-      </c>
+      <c r="C23" s="17" t="n"/>
       <c r="F23" s="6" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
           <t>收到单证日期</t>
         </is>
       </c>
-      <c r="H23" s="82" t="n">
-        <v>46198</v>
-      </c>
+      <c r="H23" s="82" t="n"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="B24" s="5" t="inlineStr">
@@ -4718,9 +4464,7 @@
           <t>货物总价</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n">
-        <v>16334.6</v>
-      </c>
+      <c r="C24" s="17" t="n"/>
       <c r="F24" s="6" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
@@ -4744,9 +4488,7 @@
           <t>进出口日期</t>
         </is>
       </c>
-      <c r="C25" s="83" t="n">
-        <v>46199</v>
-      </c>
+      <c r="C25" s="83" t="n"/>
       <c r="F25" s="6" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
@@ -4804,7 +4546,7 @@
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>示例城市</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr"/>
@@ -4995,18 +4737,14 @@
       </c>
       <c r="C45" s="22" t="inlineStr"/>
       <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="86" t="n">
-        <v>46197</v>
-      </c>
+      <c r="E45" s="86" t="n"/>
       <c r="G45" s="6" t="inlineStr">
         <is>
           <t>联系电话：</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr"/>
-      <c r="I45" s="82" t="n">
-        <v>46198</v>
-      </c>
+      <c r="I45" s="82" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="B46" s="22" t="inlineStr"/>

</xml_diff>